<commit_message>
Fix FILTER/SORTBY/HSTACK/SEQUENCE stripped on Excel open
openpyxl writes dynamic-array functions as plain text; Excel treats
them as unknown and removes them during repair. Add _xlfn._xlws.
prefix to FILTER/SORTBY and _xlfn. to HSTACK/SEQUENCE via a small
_xl() helper applied to every formula before it is written to a cell.

https://claude.ai/code/session_01EZJUaj6DYkCnAfhitpvYt3
</commit_message>
<xml_diff>
--- a/Production_Schedule.xlsx
+++ b/Production_Schedule.xlsx
@@ -1304,7 +1304,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AG$6:$AG$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AH$6:$AH$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AI$6:$AI$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AJ$6:$AJ$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AG$6:$AG$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AH$6:$AH$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AI$6:$AI$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AJ$6:$AJ$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
         <v/>
       </c>
     </row>
@@ -1462,7 +1462,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AK$6:$AK$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AL$6:$AL$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AM$6:$AM$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AN$6:$AN$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AK$6:$AK$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AL$6:$AL$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AM$6:$AM$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AN$6:$AN$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
         <v/>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AO$6:$AO$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AP$6:$AP$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AQ$6:$AQ$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AR$6:$AR$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AO$6:$AO$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AP$6:$AP$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AQ$6:$AQ$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AR$6:$AR$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
         <v/>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AS$6:$AS$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AT$6:$AT$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AU$6:$AU$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AV$6:$AV$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AS$6:$AS$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AT$6:$AT$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AU$6:$AU$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AV$6:$AV$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
         <v/>
       </c>
     </row>
@@ -1936,7 +1936,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AW$6:$AW$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AX$6:$AX$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AY$6:$AY$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AZ$6:$AZ$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AW$6:$AW$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AX$6:$AX$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AY$6:$AY$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AZ$6:$AZ$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
         <v/>
       </c>
     </row>
@@ -2094,7 +2094,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$BA$6:$BA$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$BB$6:$BB$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$BC$6:$BC$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$BD$6:$BD$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BA$6:$BA$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BB$6:$BB$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BC$6:$BC$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BD$6:$BD$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
         <v/>
       </c>
     </row>
@@ -2252,7 +2252,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$BE$6:$BE$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$BF$6:$BF$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$BG$6:$BG$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$BH$6:$BH$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BE$6:$BE$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BF$6:$BF$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BG$6:$BG$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BH$6:$BH$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
         <v/>
       </c>
     </row>
@@ -2410,7 +2410,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$BI$6:$BI$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$BJ$6:$BJ$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$BK$6:$BK$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$BL$6:$BL$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BI$6:$BI$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BJ$6:$BJ$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BK$6:$BK$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BL$6:$BL$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
         <v/>
       </c>
     </row>
@@ -8318,7 +8318,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($B$4="All",1,ISNUMBER(SEARCH($B$4,'Master Schedule'!$A$6:$A$500)))*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),FILTER('Master Schedule'!$G$6:$G$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),FILTER('Master Schedule'!$G$6:$G$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),FILTER('Master Schedule'!$L$6:$L$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1),"No jobs match")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($B$4="All",1,ISNUMBER(SEARCH($B$4,'Master Schedule'!$A$6:$A$500)))*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$G$6:$G$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$G$6:$G$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$L$6:$L$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1),"No jobs match")</f>
         <v/>
       </c>
     </row>
@@ -8477,7 +8477,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$M$6:$M$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$N$6:$N$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$O$6:$O$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$P$6:$P$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$M$6:$M$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$N$6:$N$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$O$6:$O$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$P$6:$P$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
         <v/>
       </c>
     </row>
@@ -8635,7 +8635,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$Q$6:$Q$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$R$6:$R$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$S$6:$S$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$T$6:$T$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$Q$6:$Q$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$R$6:$R$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$S$6:$S$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$T$6:$T$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
         <v/>
       </c>
     </row>
@@ -8793,7 +8793,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$U$6:$U$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$V$6:$V$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$W$6:$W$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$X$6:$X$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$U$6:$U$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$V$6:$V$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$W$6:$W$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$X$6:$X$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
         <v/>
       </c>
     </row>
@@ -8951,7 +8951,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$Y$6:$Y$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$Z$6:$Z$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AA$6:$AA$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AB$6:$AB$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$Y$6:$Y$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$Z$6:$Z$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AA$6:$AA$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AB$6:$AB$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
         <v/>
       </c>
     </row>
@@ -9109,7 +9109,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(SORTBY(HSTACK(SEQUENCE(ROWS(FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AC$6:$AC$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AD$6:$AD$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AE$6:$AE$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),FILTER('Master Schedule'!$AF$6:$AF$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AC$6:$AC$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AD$6:$AD$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AE$6:$AE$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AF$6:$AF$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace HSTACK with per-column FILTER+SORTBY in all queue sheets
HSTACK (2022+) was the real cause of the repair-on-open failure:
openpyxl cannot reliably write it, and even with the _xlfn prefix
it is unavailable in older Excel 365 channels, causing IFERROR to
swallow the entire formula silently.

New approach: each column in the data area (A8:L8 for station queues,
A8:K8 for Queue-All) gets its own SORTBY(FILTER(...)) formula. All
columns share the same condition and sort keys (Priority Rank, then
Due Date) so row ordering is identical across columns. No HSTACK
or 2D spill needed. Also corrects the SEQUENCE prefix to
_xlfn._xlws.SEQUENCE (dynamic-array namespace).

https://claude.ai/code/session_01EZJUaj6DYkCnAfhitpvYt3
</commit_message>
<xml_diff>
--- a/Production_Schedule.xlsx
+++ b/Production_Schedule.xlsx
@@ -1304,7 +1304,51 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AG$6:$AG$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AH$6:$AH$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AI$6:$AI$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AJ$6:$AJ$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AG$6:$AG$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AH$6:$AH$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AI$6:$AI$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AJ$6:$AJ$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AG$6:$AG$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
     </row>
@@ -1462,7 +1506,51 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AK$6:$AK$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AL$6:$AL$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AM$6:$AM$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AN$6:$AN$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AK$6:$AK$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AL$6:$AL$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AM$6:$AM$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AN$6:$AN$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AK$6:$AK$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
     </row>
@@ -1620,7 +1708,51 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AO$6:$AO$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AP$6:$AP$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AQ$6:$AQ$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AR$6:$AR$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AO$6:$AO$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AP$6:$AP$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AQ$6:$AQ$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AR$6:$AR$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AO$6:$AO$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
     </row>
@@ -1778,7 +1910,51 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AS$6:$AS$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AT$6:$AT$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AU$6:$AU$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AV$6:$AV$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AS$6:$AS$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AT$6:$AT$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AU$6:$AU$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AV$6:$AV$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AS$6:$AS$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
     </row>
@@ -1936,7 +2112,51 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AW$6:$AW$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AX$6:$AX$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AY$6:$AY$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AZ$6:$AZ$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AW$6:$AW$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AX$6:$AX$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AY$6:$AY$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AZ$6:$AZ$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AW$6:$AW$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
     </row>
@@ -2094,7 +2314,51 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BA$6:$BA$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BB$6:$BB$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BC$6:$BC$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BD$6:$BD$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$BA$6:$BA$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$BB$6:$BB$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$BC$6:$BC$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$BD$6:$BD$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BA$6:$BA$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
     </row>
@@ -2252,7 +2516,51 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BE$6:$BE$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BF$6:$BF$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BG$6:$BG$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BH$6:$BH$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$BE$6:$BE$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$BF$6:$BF$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$BG$6:$BG$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$BH$6:$BH$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BE$6:$BE$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
     </row>
@@ -2410,7 +2718,51 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BI$6:$BI$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BJ$6:$BJ$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BK$6:$BK$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$BL$6:$BL$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$BI$6:$BI$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$BJ$6:$BJ$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$BK$6:$BK$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$BL$6:$BL$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$BI$6:$BI$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
     </row>
@@ -8318,7 +8670,47 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($B$4="All",1,ISNUMBER(SEARCH($B$4,'Master Schedule'!$A$6:$A$500)))*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$G$6:$G$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$G$6:$G$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$L$6:$L$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1),"No jobs match")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$G$6:$G$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$G$6:$G$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$L$6:$L$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$A$6:$A$500&lt;&gt;"")*IF($D$4="All",1,'Master Schedule'!$F$6:$F$500=$D$4)),1),"")</f>
         <v/>
       </c>
     </row>
@@ -8477,7 +8869,51 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$M$6:$M$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$N$6:$N$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$O$6:$O$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$P$6:$P$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$M$6:$M$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$N$6:$N$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$O$6:$O$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$P$6:$P$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$M$6:$M$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
     </row>
@@ -8635,7 +9071,51 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$Q$6:$Q$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$R$6:$R$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$S$6:$S$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$T$6:$T$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$Q$6:$Q$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$R$6:$R$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$S$6:$S$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$T$6:$T$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Q$6:$Q$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
     </row>
@@ -8793,7 +9273,51 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$U$6:$U$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$V$6:$V$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$W$6:$W$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$X$6:$X$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$U$6:$U$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$V$6:$V$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$W$6:$W$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$X$6:$X$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$U$6:$U$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
     </row>
@@ -8951,7 +9475,51 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$Y$6:$Y$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$Z$6:$Z$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AA$6:$AA$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AB$6:$AB$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$Y$6:$Y$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$Z$6:$Z$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AA$6:$AA$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AB$6:$AB$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$Y$6:$Y$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
     </row>
@@ -9109,7 +9677,51 @@
     </row>
     <row r="8">
       <c r="A8">
-        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn.HSTACK(_xlfn.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AC$6:$AC$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AD$6:$AD$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AE$6:$AE$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$AF$6:$AF$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;""))),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"No jobs in queue")</f>
+        <f>IFERROR(_xlfn._xlws.SEQUENCE(ROWS(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")))),"")</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$A$6:$A$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$B$6:$B$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$C$6:$C$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$E$6:$E$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$F$6:$F$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$J$6:$J$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AC$6:$AC$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AD$6:$AD$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AE$6:$AE$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IFERROR(_xlfn._xlws.SORTBY(_xlfn._xlws.FILTER('Master Schedule'!$AF$6:$AF$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),_xlfn._xlws.FILTER('Master Schedule'!$K$6:$K$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1,_xlfn._xlws.FILTER('Master Schedule'!$H$6:$H$500,('Master Schedule'!$AC$6:$AC$500&lt;&gt;"Not Started")*('Master Schedule'!$A$6:$A$500&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>